<commit_message>
Workbook: Ledger sheet section C, the euro-portfolio position as formulas
Below section B: the one buy row with a rate column, the position in
euros, and the valuation with the AAPL close taken from Positions and the
spot rate typed. Blue inputs, black formulas, the hand-computed Part 8 C
figures stated in the last row. Written with openpyxl, not recalculated
here; Excel computes on opening.
</commit_message>
<xml_diff>
--- a/tests/golden/expected_values.xlsx
+++ b/tests/golden/expected_values.xlsx
@@ -24389,7 +24389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="51" min="1" max="1"/>
@@ -25335,6 +25335,223 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="100" t="inlineStr">
+        <is>
+          <t>C. One foreign-currency position in a euro portfolio — D15–D18. Base currency EUR; AAPL quoted in USD; rates are EUR per USD, stated and synthetic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="100" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B44" s="100" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C44" s="100" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D44" s="100" t="inlineStr">
+        <is>
+          <t>Price (USD)</t>
+        </is>
+      </c>
+      <c r="E44" s="100" t="inlineStr">
+        <is>
+          <t>Rate EUR/USD</t>
+        </is>
+      </c>
+      <c r="F44" s="100" t="inlineStr">
+        <is>
+          <t>Fees (EUR)</t>
+        </is>
+      </c>
+      <c r="G44" s="100" t="inlineStr">
+        <is>
+          <t>Amount (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="101" t="inlineStr">
+        <is>
+          <t>2024-02-20</t>
+        </is>
+      </c>
+      <c r="B45" s="101" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C45" s="101" t="n">
+        <v>100</v>
+      </c>
+      <c r="D45" s="101" t="n">
+        <v>200</v>
+      </c>
+      <c r="E45" s="101" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F45" s="101" t="n">
+        <v>5</v>
+      </c>
+      <c r="G45">
+        <f>IF(B45="buy",C45*D45*E45+F45,C45*D45*E45-F45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="100" t="inlineStr">
+        <is>
+          <t>Position after (D13, D18: in EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="100" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="B48">
+        <f>C45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="100" t="inlineStr">
+        <is>
+          <t>Cost basis (EUR)</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>G45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="100" t="inlineStr">
+        <is>
+          <t>Average (EUR)</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>B49/B48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="100" t="inlineStr">
+        <is>
+          <t>First buy</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>A45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="100" t="inlineStr">
+        <is>
+          <t>Valuation (D16, D17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="100" t="inlineStr">
+        <is>
+          <t>Price now (USD)</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>Positions!G6</f>
+        <v/>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AAPL close 2026-09-02, from Positions</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="100" t="inlineStr">
+        <is>
+          <t>Spot EUR/USD</t>
+        </is>
+      </c>
+      <c r="B55" s="101" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>stated, as of 2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="100" t="inlineStr">
+        <is>
+          <t>Market value (EUR)</t>
+        </is>
+      </c>
+      <c r="B56">
+        <f>B48*B54*B55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="100" t="inlineStr">
+        <is>
+          <t>P&amp;L abs (EUR)</t>
+        </is>
+      </c>
+      <c r="B57">
+        <f>B56-B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="100" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="B58">
+        <f>B57/B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="100" t="inlineStr">
+        <is>
+          <t>USD P&amp;L % for contrast</t>
+        </is>
+      </c>
+      <c r="B59">
+        <f>(B48*B54-B48*D45)/(B48*D45)</f>
+        <v/>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>the price part alone; the split is not computed (Part 8 C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Hand-computed (expected_values.md Part 8 C): amount 18,405.00; 100 @ 184.05 EUR; at 324.96 USD and 0.8500, market value 27,621.60, P&amp;L +9,216.60 (+50.08%); in USD +62.48%.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add the Prices sheet, Part 9, to the workbook
</commit_message>
<xml_diff>
--- a/tests/golden/expected_values.xlsx
+++ b/tests/golden/expected_values.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -25402,7 +25403,7 @@
       <c r="F45" s="101" t="n">
         <v>5</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="50">
         <f>IF(B45="buy",C45*D45*E45+F45,C45*D45*E45-F45)</f>
         <v/>
       </c>
@@ -25420,7 +25421,7 @@
           <t>Qty</t>
         </is>
       </c>
-      <c r="B48">
+      <c r="B48" s="50">
         <f>C45</f>
         <v/>
       </c>
@@ -25431,7 +25432,7 @@
           <t>Cost basis (EUR)</t>
         </is>
       </c>
-      <c r="B49">
+      <c r="B49" s="50">
         <f>G45</f>
         <v/>
       </c>
@@ -25442,7 +25443,7 @@
           <t>Average (EUR)</t>
         </is>
       </c>
-      <c r="B50">
+      <c r="B50" s="50">
         <f>B49/B48</f>
         <v/>
       </c>
@@ -25453,7 +25454,7 @@
           <t>First buy</t>
         </is>
       </c>
-      <c r="B51">
+      <c r="B51" s="50">
         <f>A45</f>
         <v/>
       </c>
@@ -25471,11 +25472,11 @@
           <t>Price now (USD)</t>
         </is>
       </c>
-      <c r="B54">
+      <c r="B54" s="50">
         <f>Positions!G6</f>
         <v/>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="50" t="inlineStr">
         <is>
           <t>AAPL close 2026-09-02, from Positions</t>
         </is>
@@ -25490,7 +25491,7 @@
       <c r="B55" s="101" t="n">
         <v>0.85</v>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="50" t="inlineStr">
         <is>
           <t>stated, as of 2026-09-02</t>
         </is>
@@ -25502,7 +25503,7 @@
           <t>Market value (EUR)</t>
         </is>
       </c>
-      <c r="B56">
+      <c r="B56" s="50">
         <f>B48*B54*B55</f>
         <v/>
       </c>
@@ -25513,7 +25514,7 @@
           <t>P&amp;L abs (EUR)</t>
         </is>
       </c>
-      <c r="B57">
+      <c r="B57" s="50">
         <f>B56-B49</f>
         <v/>
       </c>
@@ -25524,7 +25525,7 @@
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="B58">
+      <c r="B58" s="50">
         <f>B57/B49</f>
         <v/>
       </c>
@@ -25535,20 +25536,435 @@
           <t>USD P&amp;L % for contrast</t>
         </is>
       </c>
-      <c r="B59">
+      <c r="B59" s="50">
         <f>(B48*B54-B48*D45)/(B48*D45)</f>
         <v/>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="50" t="inlineStr">
         <is>
           <t>the price part alone; the split is not computed (Part 8 C)</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="50" t="inlineStr">
         <is>
           <t>Hand-computed (expected_values.md Part 8 C): amount 18,405.00; 100 @ 184.05 EUR; at 324.96 USD and 0.8500, market value 27,621.60, P&amp;L +9,216.60 (+50.08%); in USD +62.48%.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="51" min="1" max="1"/>
+    <col width="20" customWidth="1" style="51" min="2" max="2"/>
+    <col width="18" customWidth="1" style="51" min="3" max="3"/>
+    <col width="18" customWidth="1" style="51" min="4" max="4"/>
+    <col width="20" customWidth="1" style="51" min="5" max="5"/>
+    <col width="20" customWidth="1" style="51" min="6" max="6"/>
+    <col width="22" customWidth="1" style="51" min="7" max="7"/>
+    <col width="32" customWidth="1" style="51" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>Part 9 — The price source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Decisions D19–D20: a close is the exchange's as-traded print, split-adjusted only; when two sources disagree the exchange's print wins and nothing averages. Blue = typed from the exchange's own historical quotes (api.nasdaq.com, Close/Last), fetched 2026-09-10; black = formula. Tolerance: equal after rounding to the cent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="100" t="inlineStr">
+        <is>
+          <t>A. The valuation date, 2026-09-02 — the exchange against Positions!G (Part 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="100" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B5" s="100" t="inlineStr">
+        <is>
+          <t>Exchange 2026-09-02</t>
+        </is>
+      </c>
+      <c r="C5" s="100" t="inlineStr">
+        <is>
+          <t>Part 1 (Positions)</t>
+        </is>
+      </c>
+      <c r="D5" s="100" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="B6" s="101" t="n">
+        <v>765.16</v>
+      </c>
+      <c r="C6">
+        <f>Positions!G5</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>ROUND(C6,2)-ROUND(B6,2)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>IF(ABS(D6)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B7" s="101" t="n">
+        <v>324.96</v>
+      </c>
+      <c r="C7">
+        <f>Positions!G6</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>ROUND(C7,2)-ROUND(B7,2)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>IF(ABS(D7)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B8" s="101" t="n">
+        <v>496.82</v>
+      </c>
+      <c r="C8">
+        <f>Positions!G7</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>ROUND(C8,2)-ROUND(B8,2)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IF(ABS(D8)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B9" s="101" t="n">
+        <v>275.21</v>
+      </c>
+      <c r="C9">
+        <f>Positions!G8</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>ROUND(C9,2)-ROUND(B9,2)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>IF(ABS(D9)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B10" s="101" t="n">
+        <v>356.22</v>
+      </c>
+      <c r="C10">
+        <f>Positions!G9</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>ROUND(C10,2)-ROUND(B10,2)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>IF(ABS(D10)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="B11" s="101" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="C11">
+        <f>Positions!G10</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>ROUND(C11,2)-ROUND(B11,2)</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>IF(ABS(D11)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TLT</t>
+        </is>
+      </c>
+      <c r="B12" s="101" t="n">
+        <v>81.95</v>
+      </c>
+      <c r="C12">
+        <f>Positions!G11</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>ROUND(C12,2)-ROUND(B12,2)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>IF(ABS(D12)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="B13" s="101" t="n">
+        <v>402.78</v>
+      </c>
+      <c r="C13">
+        <f>Positions!G12</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>ROUND(C13,2)-ROUND(B13,2)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>IF(ABS(D13)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VNQ</t>
+        </is>
+      </c>
+      <c r="B14" s="101" t="n">
+        <v>95.78</v>
+      </c>
+      <c r="C14">
+        <f>Positions!G13</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>ROUND(C14,2)-ROUND(B14,2)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>IF(ABS(D14)&lt;0.005,"agrees","DISAGREES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agreeing</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(E6:E14,"agrees")</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="100" t="inlineStr">
+        <is>
+          <t>B. Dates before a dividend — the falsifier. The committed series is benchmark_closes.csv (Part 4's 252 closes); the database column is data/portfolio.db as read on 2026-09-10, after the provider had refetched with its default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="100" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B18" s="100" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C18" s="100" t="inlineStr">
+        <is>
+          <t>Exchange</t>
+        </is>
+      </c>
+      <c r="D18" s="100" t="inlineStr">
+        <is>
+          <t>Committed series</t>
+        </is>
+      </c>
+      <c r="E18" s="100" t="inlineStr">
+        <is>
+          <t>Database 2026-09-10</t>
+        </is>
+      </c>
+      <c r="F18" s="100" t="inlineStr">
+        <is>
+          <t>Series minus exchange</t>
+        </is>
+      </c>
+      <c r="G18" s="100" t="inlineStr">
+        <is>
+          <t>Database minus exchange</t>
+        </is>
+      </c>
+      <c r="H18" s="100" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C19" s="101" t="n">
+        <v>270.24</v>
+      </c>
+      <c r="D19" s="101" t="n">
+        <v>270.24</v>
+      </c>
+      <c r="E19" s="101" t="n">
+        <v>268.9137</v>
+      </c>
+      <c r="F19">
+        <f>ROUND(D19,2)-ROUND(C19,2)</f>
+        <v/>
+      </c>
+      <c r="G19">
+        <f>ROUND(E19,2)-ROUND(C19,2)</f>
+        <v/>
+      </c>
+      <c r="H19">
+        <f>IF(ABS(G19)&lt;0.005,"database agrees",IF(ABS(F19)&lt;0.005,"database wrong, series is the print","both differ"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TLT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C20" s="101" t="n">
+        <v>82.88</v>
+      </c>
+      <c r="D20" s="101" t="n">
+        <v>82.88</v>
+      </c>
+      <c r="E20" s="101" t="n">
+        <v>82.56359999999999</v>
+      </c>
+      <c r="F20">
+        <f>ROUND(D20,2)-ROUND(C20,2)</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>ROUND(E20,2)-ROUND(C20,2)</f>
+        <v/>
+      </c>
+      <c r="H20">
+        <f>IF(ABS(G20)&lt;0.005,"database agrees",IF(ABS(F20)&lt;0.005,"database wrong, series is the print","both differ"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Over the whole fetch (20 August to 3 September, 99 rows): 90 rows lie inside the committed series and all 90 agree to the cent; the database agrees on 82 and is lower on 17, every one a JNJ, NEE or TLT row before that holding's latest ex-dividend date. Cause: the provider's history call uses the library default, which returns the dividend-adjusted close. Fix at the provider; the reference does not move (D20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Hand-computed (expected_values.md Part 9): nine of nine on 2026-09-02; JNJ 2026-08-21 database 268.91 against the print 270.24; TLT 2026-08-28 82.56 against 82.88.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: the Filed column on the Philosophy sheet, formulas shifted with it
</commit_message>
<xml_diff>
--- a/tests/golden/expected_values.xlsx
+++ b/tests/golden/expected_values.xlsx
@@ -963,7 +963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -990,7 +990,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Synthetic figures for candidate W-1 (docs/WATCHLIST.md), typed inputs in bold as on the Compliance sheet; everything else computes. Reference for the checker's arithmetic, not for the company. As-of 2026-09-10; FY2021 to FY2025 reported by then (D21).</t>
+          <t>Synthetic figures for candidate W-1 (docs/WATCHLIST.md), typed inputs in bold as on the Compliance sheet; everything else computes. Reference for the checker's arithmetic, not for the company. As-of 2026-09-10; FY2021 to FY2025 reported by then (D21). Filed dates are synthetic, about five weeks after each year end; D21 counts a year by them.</t>
         </is>
       </c>
     </row>
@@ -1028,50 +1028,55 @@
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
+          <t>Filed</t>
+        </is>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="D7" s="40" t="inlineStr">
+      <c r="E7" s="40" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="E7" s="40" t="inlineStr">
+      <c r="F7" s="40" t="inlineStr">
         <is>
           <t>Operating income</t>
         </is>
       </c>
-      <c r="F7" s="40" t="inlineStr">
+      <c r="G7" s="40" t="inlineStr">
         <is>
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="G7" s="40" t="inlineStr">
+      <c r="H7" s="40" t="inlineStr">
         <is>
           <t>D&amp;A</t>
         </is>
       </c>
-      <c r="H7" s="40" t="inlineStr">
+      <c r="I7" s="40" t="inlineStr">
         <is>
           <t>Operating cash flow</t>
         </is>
       </c>
-      <c r="I7" s="40" t="inlineStr">
+      <c r="J7" s="40" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="J7" s="40" t="inlineStr">
+      <c r="K7" s="40" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="K7" s="40" t="inlineStr">
+      <c r="L7" s="40" t="inlineStr">
         <is>
           <t>Debt</t>
         </is>
       </c>
-      <c r="L7" s="40" t="inlineStr">
+      <c r="M7" s="40" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
@@ -1088,19 +1093,24 @@
           <t>2021-12-31</t>
         </is>
       </c>
-      <c r="E8" s="40" t="n">
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>2022-02-04</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="n">
         <v>20000</v>
       </c>
-      <c r="F8" s="40" t="n">
+      <c r="G8" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="J8" s="40" t="n">
+      <c r="K8" s="40" t="n">
         <v>120000</v>
       </c>
-      <c r="K8" s="40" t="n">
+      <c r="L8" s="40" t="n">
         <v>20000</v>
       </c>
-      <c r="L8" s="40" t="n">
+      <c r="M8" s="40" t="n">
         <v>40000</v>
       </c>
     </row>
@@ -1115,19 +1125,24 @@
           <t>2022-12-31</t>
         </is>
       </c>
-      <c r="E9" s="40" t="n">
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>2023-02-03</t>
+        </is>
+      </c>
+      <c r="F9" s="40" t="n">
         <v>13500</v>
       </c>
-      <c r="F9" s="40" t="n">
+      <c r="G9" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="J9" s="40" t="n">
+      <c r="K9" s="40" t="n">
         <v>128000</v>
       </c>
-      <c r="K9" s="40" t="n">
+      <c r="L9" s="40" t="n">
         <v>22000</v>
       </c>
-      <c r="L9" s="40" t="n">
+      <c r="M9" s="40" t="n">
         <v>42000</v>
       </c>
     </row>
@@ -1142,25 +1157,30 @@
           <t>2023-12-31</t>
         </is>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>2024-02-02</t>
+        </is>
+      </c>
+      <c r="D10" s="40" t="n">
         <v>100000</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="E10" s="40" t="n">
         <v>55000</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="F10" s="40" t="n">
         <v>24000</v>
       </c>
-      <c r="F10" s="40" t="n">
+      <c r="G10" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="J10" s="40" t="n">
+      <c r="K10" s="40" t="n">
         <v>140000</v>
       </c>
-      <c r="K10" s="40" t="n">
+      <c r="L10" s="40" t="n">
         <v>20000</v>
       </c>
-      <c r="L10" s="40" t="n">
+      <c r="M10" s="40" t="n">
         <v>40000</v>
       </c>
     </row>
@@ -1175,25 +1195,30 @@
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="C11" s="40" t="n">
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>2025-02-05</t>
+        </is>
+      </c>
+      <c r="D11" s="40" t="n">
         <v>112000</v>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="E11" s="40" t="n">
         <v>63840</v>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="F11" s="40" t="n">
         <v>30000</v>
       </c>
-      <c r="F11" s="40" t="n">
+      <c r="G11" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="J11" s="40" t="n">
+      <c r="K11" s="40" t="n">
         <v>150000</v>
       </c>
-      <c r="K11" s="40" t="n">
+      <c r="L11" s="40" t="n">
         <v>18000</v>
       </c>
-      <c r="L11" s="40" t="n">
+      <c r="M11" s="40" t="n">
         <v>43000</v>
       </c>
     </row>
@@ -1208,34 +1233,39 @@
           <t>2025-12-31</t>
         </is>
       </c>
-      <c r="C12" s="40" t="n">
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="D12" s="40" t="n">
         <v>125000</v>
       </c>
-      <c r="D12" s="40" t="n">
+      <c r="E12" s="40" t="n">
         <v>72500</v>
       </c>
-      <c r="E12" s="40" t="n">
+      <c r="F12" s="40" t="n">
         <v>36000</v>
       </c>
-      <c r="F12" s="40" t="n">
+      <c r="G12" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="G12" s="40" t="n">
+      <c r="H12" s="40" t="n">
         <v>16000</v>
       </c>
-      <c r="H12" s="40" t="n">
+      <c r="I12" s="40" t="n">
         <v>52780</v>
       </c>
-      <c r="I12" s="40" t="n">
+      <c r="J12" s="40" t="n">
         <v>22000</v>
       </c>
-      <c r="J12" s="40" t="n">
+      <c r="K12" s="40" t="n">
         <v>170000</v>
       </c>
-      <c r="K12" s="40" t="n">
+      <c r="L12" s="40" t="n">
         <v>16000</v>
       </c>
-      <c r="L12" s="40" t="n">
+      <c r="M12" s="40" t="n">
         <v>42000</v>
       </c>
     </row>
@@ -1319,11 +1349,11 @@
         <v/>
       </c>
       <c r="B21">
-        <f>J8+K8-L8</f>
+        <f>K8+L8-M8</f>
         <v/>
       </c>
       <c r="C21">
-        <f>E8*(1-F8)</f>
+        <f>F8*(1-G8)</f>
         <v/>
       </c>
       <c r="D21">
@@ -1337,11 +1367,11 @@
         <v/>
       </c>
       <c r="B22">
-        <f>J9+K9-L9</f>
+        <f>K9+L9-M9</f>
         <v/>
       </c>
       <c r="C22">
-        <f>E9*(1-F9)</f>
+        <f>F9*(1-G9)</f>
         <v/>
       </c>
       <c r="D22">
@@ -1355,11 +1385,11 @@
         <v/>
       </c>
       <c r="B23">
-        <f>J10+K10-L10</f>
+        <f>K10+L10-M10</f>
         <v/>
       </c>
       <c r="C23">
-        <f>E10*(1-F10)</f>
+        <f>F10*(1-G10)</f>
         <v/>
       </c>
       <c r="D23">
@@ -1367,7 +1397,7 @@
         <v/>
       </c>
       <c r="E23">
-        <f>D10/C10</f>
+        <f>E10/D10</f>
         <v/>
       </c>
     </row>
@@ -1377,11 +1407,11 @@
         <v/>
       </c>
       <c r="B24">
-        <f>J11+K11-L11</f>
+        <f>K11+L11-M11</f>
         <v/>
       </c>
       <c r="C24">
-        <f>E11*(1-F11)</f>
+        <f>F11*(1-G11)</f>
         <v/>
       </c>
       <c r="D24">
@@ -1389,7 +1419,7 @@
         <v/>
       </c>
       <c r="E24">
-        <f>D11/C11</f>
+        <f>E11/D11</f>
         <v/>
       </c>
     </row>
@@ -1399,11 +1429,11 @@
         <v/>
       </c>
       <c r="B25">
-        <f>J12+K12-L12</f>
+        <f>K12+L12-M12</f>
         <v/>
       </c>
       <c r="C25">
-        <f>E12*(1-F12)</f>
+        <f>F12*(1-G12)</f>
         <v/>
       </c>
       <c r="D25">
@@ -1411,10 +1441,11 @@
         <v/>
       </c>
       <c r="E25">
-        <f>D12/C12</f>
-        <v/>
-      </c>
-    </row>
+        <f>E12/D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -1422,7 +1453,7 @@
         </is>
       </c>
       <c r="B27">
-        <f>K12-L12</f>
+        <f>L12-M12</f>
         <v/>
       </c>
     </row>
@@ -1433,7 +1464,7 @@
         </is>
       </c>
       <c r="B28">
-        <f>E12+G12</f>
+        <f>F12+H12</f>
         <v/>
       </c>
     </row>
@@ -1455,7 +1486,7 @@
         </is>
       </c>
       <c r="B30">
-        <f>H12-I12</f>
+        <f>I12-J12</f>
         <v/>
       </c>
     </row>
@@ -1492,6 +1523,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="40" t="inlineStr">
         <is>
@@ -1668,6 +1700,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="40" t="inlineStr">
         <is>
@@ -1915,6 +1948,7 @@
         <v/>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -1937,6 +1971,7 @@
         <v/>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="40" t="inlineStr">
         <is>
@@ -1997,6 +2032,7 @@
         <v/>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>

</xml_diff>